<commit_message>
Update content-calendar: Topic 4 scheduled
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -1913,7 +1913,32 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>why-worklife, worklife-lessons, start-here-worklife</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Podcast Rec topic. 27 posts scheduled Apr 4-27.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 3 Working Genius
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -2108,7 +2108,32 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>6-types-of-working-genius, why-your-team-feels-stuck, genius-competency-frustration</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>3 carousels, 27 posts scheduled. Footer: Certified Working Genius Facilitator | Author</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 4 Five Dysfunctions
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -2150,7 +2150,32 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>five-dysfunctions-overview, signs-team-dysfunctional, building-cohesive-team</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>3 carousels, 27 posts scheduled. Footer: Leadership Team Facilitator | Keynote Speaker | Author</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Topic 3 Crucial Conversations done
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -59,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1871,7 +1874,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Carousel Created</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1881,22 +1884,22 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>priorities-just-words, why-teams-repeat, break-the-cycle</t>
+          <t>why-priorities-fail, signs-plan-will-fail, break-the-cycle</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>8, 8, 8</t>
+          <t>8, 7, 8</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky (carousel 3: 5 platforms failed duplicate detection)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Pain Point topic. 27 posts scheduled Apr 1-24.</t>
+          <t>Pain point topic. 3 carousels. Carousel 3 blocked by Buffer duplicate detection on LI/FB/Threads/X/Bluesky.</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1916,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Carousel Created</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1923,22 +1926,22 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>why-worklife, worklife-lessons, start-here-worklife</t>
+          <t>worklife-podcast-rec, worklife-why-listen</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>8, 8, 8</t>
+          <t>8, 7</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Podcast Rec topic. 27 posts scheduled Apr 4-27.</t>
+          <t>2 carousels. All 9 platforms scheduled successfully.</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1958,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>No testimonial content found online. Needs manual input of testimonial text.</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1980,32 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>keynote-speaking-service, why-book-jonno</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2 carousels. All 9 platforms scheduled successfully.</t>
         </is>
       </c>
     </row>
@@ -1989,7 +2022,32 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>asba-93-percent-proof, asba-what-makes-pd-great</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2 carousels. YouTube and Google Business disconnected. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2064,32 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>exec-team-dysfunction, fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>9, 7</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2 carousels. All 9 platforms scheduled successfully. Based on Lencioni's Five Dysfunctions.</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2106,32 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>extreme-ownership-why-read, extreme-ownership-principles, extreme-ownership-apply</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>8, 8, 7</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>3 carousels. YouTube and Google Business disconnected. Pinterest skipped.</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2148,32 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>perfect-meeting-danger, perfect-meeting-fix</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Pain point topic. YouTube/Google Business disconnected. TikTok scheduled May 25-26.</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2190,32 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>learning-leader-rec, learning-leader-lessons</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Podcast rec for Ryan Hawk. YouTube/Google Business disconnected. TikTok scheduled May 27-28.</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2232,30 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>offsite-insights-edward-amey, leadership-disability-edward-amey</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>No specific testimonial quote found. Built carousels from verified podcast content (EP225) and public bio.</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2272,30 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>why-leaders-need-a-coach, what-coaching-looks-like, cost-of-no-coach</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Service promo carousel. No people tagged.</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2322,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>6-types-of-working-genius, why-your-team-feels-stuck, genius-competency-frustration</t>
+          <t>wg-6-types, wg-genius-or-frustration, wg-transforms-teams</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2133,7 +2337,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>3 carousels, 27 posts scheduled. Footer: Certified Working Genius Facilitator | Author</t>
+          <t>All 9 platforms scheduled. YouTube on Apr 15-17 due to daily limits.</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2364,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>five-dysfunctions-overview, signs-team-dysfunctional, building-cohesive-team</t>
+          <t>5d-overview, 5d-overcome, 5d-warning-signs</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2175,7 +2379,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>3 carousels, 27 posts scheduled. Footer: Leadership Team Facilitator | Keynote Speaker | Author</t>
+          <t>All 9 platforms scheduled. YouTube on Apr 18-20.</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2396,32 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>crucial-conversations-overview, crucial-conversations-state-method, crucial-conversations-crib-technique</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>6, 7, 7</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>3 carousels: book overview, STATE method, CRIB technique. 27 posts scheduled.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Topic 4 done, all 4 topics complete
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -2438,7 +2438,32 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>best-teacher-resigned-warning-signs, best-teacher-resigned-why-they-leave, best-teacher-resigned-how-to-keep</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>6, 6, 7</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>3 carousels: warning signs, why they leave, how to keep them. 27 posts scheduled.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx — session 2026-03-27 (4 topics)
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -2396,7 +2396,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Carousel Created</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2406,22 +2406,22 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>crucial-conversations-overview, crucial-conversations-state-method, crucial-conversations-crib-technique</t>
+          <t>crucial-conversations-why-read, crucial-conversations-7-skills, crucial-conversations-apply</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>6, 7, 7</t>
+          <t>8, 9, 8</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>3 carousels: book overview, STATE method, CRIB technique. 27 posts scheduled.</t>
+          <t>Book rec. 3 carousels. All 9 platforms. YouTube Apr 28-30. TikTok Jun 9-11. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Carousel Created</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2448,22 +2448,22 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>best-teacher-resigned-warning-signs, best-teacher-resigned-why-they-leave, best-teacher-resigned-how-to-keep</t>
+          <t>teacher-resigned-what-happened, teacher-resigned-warning-signs, teacher-resigned-how-to-keep</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>6, 6, 7</t>
+          <t>8, 8, 8</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, TikTok, Threads, YouTube, Google Business, X/Twitter, Bluesky</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>3 carousels: warning signs, why they leave, how to keep them. 27 posts scheduled.</t>
+          <t>Pain point. 3 carousels. All 9 platforms. YouTube May 1-3. TikTok Jun 12-14. Pinterest skipped.</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,32 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>dare-to-lead-why-listen, dare-to-lead-key-themes</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Podcast rec. 2 carousels. All 9 platforms. YouTube May 4-5. TikTok Jun 15-16. Pinterest skipped.</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2522,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>No testimonial content found online. Needs manual input of testimonial text.</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2544,32 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>board-offsite-why, board-offsite-5-signs</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Service topic. No blog URL. 2 carousels. Tim Chalmers row skipped (no content found).</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2586,32 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>pre-brief-call, 5-questions-before-offsite</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Behind the scenes content. No people to tag.</t>
         </is>
       </c>
     </row>
@@ -2541,6 +2621,11 @@
           <t>Vulnerability-Based Trust</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2548,7 +2633,32 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>what-is-vulnerability-based-trust, 7-ways-vulnerability-trust, leader-must-go-first</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>8, 9, 8</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Blog post carousel. 3 carousels from Lencioni VBT concept.</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2675,32 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>atomic-habits-book-rec, 4-laws-behaviour-change</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Book rec. James Clear tagged. Footer: Author | Keynote Speaker</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2717,27 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>offsite-nothing-changed, 3-signs-offsite-fail</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update carousel-data/content-calendar.xlsx - 2026-03-27 carousel run
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -18,9 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -61,12 +59,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1373,32 +1370,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Why Listen to Craig Groeschel, 5 Key Themes, 3 Reasons to Subscribe</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>8, 7, 6</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Pinterest skipped (no boards)</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1415,32 +1387,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>asba-working-genius-in-action, asba-93-percent-rated-excellent, asba-what-school-leaders-took-away</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>7, 7, 7</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>3 carousels from ASBA testimonial. TikTok/YouTube hit daily Buffer limits. Pinterest skipped (no boards).</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1457,32 +1404,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>offsite-why-your-team-needs-one, offsite-what-to-expect, offsite-common-mistakes, offsite-book-your-offsite</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>8, 8, 8, 7</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>4 carousels from service page. Pinterest skipped (no boards). YouTube Apr 11-14. TikTok May 8-11.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1499,32 +1421,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>5-dysfunctions-overview, 5-dysfunctions-trust-conflict, 5-dysfunctions-commitment-results, 5-dysfunctions-action-plan</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>9, 8, 9, 8</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>4 carousels from framework topic. Pinterest skipped (no boards).</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1541,32 +1438,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>imposter-syndrome-signs, imposter-syndrome-cost, imposter-syndrome-overcome</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>8, 8, 8</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>3 carousels from blog topic. Pinterest skipped.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1583,32 +1455,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>unreasonable-hospitality-why-read, unreasonable-hospitality-lessons, unreasonable-hospitality-apply</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>7, 7, 7</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>3 carousels from book rec. Pinterest skipped.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1625,32 +1472,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>losing-teachers-warning-signs, losing-teachers-real-reasons, losing-teachers-what-to-do</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>8, 8, 7</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>3 carousels from pain point topic. Pinterest skipped.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1667,32 +1489,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>hbr-ideacast-why-listen, hbr-ideacast-key-themes, hbr-ideacast-reasons-subscribe</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>8, 7, 6</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>3 carousels from podcast rec. Pinterest skipped (no boards).</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1709,17 +1506,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>redlands-wg-overview, redlands-wg-discoveries, redlands-wg-book-session</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1736,17 +1523,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>schools-wg-why, schools-wg-how, schools-wg-transform</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1763,17 +1540,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>wg-session-inside, wg-session-moments, wg-session-book</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1790,32 +1557,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>understanding-uncertainty, decision-making-uncertainty, communication-trust-uncertainty, resilience-adaptive-strategy</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>8, 8, 8, 8</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>4 carousels from blog post. All 9 platforms scheduled. YouTube Apr 15-18. TikTok Mar 30-31.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1832,32 +1574,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>radical-candor-why-read, radical-candor-four-quadrants, radical-candor-in-practice</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>8, 8, 8</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>3 carousels from book rec. All 9 platforms. YouTube Apr 19-21. TikTok Apr 1-2.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1874,32 +1591,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>why-priorities-fail, signs-plan-will-fail, break-the-cycle</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>8, 7, 8</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky (carousel 3: 5 platforms failed duplicate detection)</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Pain point topic. 3 carousels. Carousel 3 blocked by Buffer duplicate detection on LI/FB/Threads/X/Bluesky.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1916,32 +1608,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>worklife-podcast-rec, worklife-why-listen</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>8, 7</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>2 carousels. All 9 platforms scheduled successfully.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1958,12 +1625,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Skipped</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>No testimonial content found online. Needs manual input of testimonial text.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1980,32 +1642,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>keynote-speaking-service, why-book-jonno</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>8, 7</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>2 carousels. All 9 platforms scheduled successfully.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2022,32 +1659,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>asba-93-percent-proof, asba-what-makes-pd-great</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>8, 8</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>2 carousels. YouTube and Google Business disconnected. Pinterest skipped (no boards).</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2064,32 +1676,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>exec-team-dysfunction, fix-dysfunctional-team</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>9, 7</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>2 carousels. All 9 platforms scheduled successfully. Based on Lencioni's Five Dysfunctions.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2106,32 +1693,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>extreme-ownership-why-read, extreme-ownership-principles, extreme-ownership-apply</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>8, 8, 7</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>3 carousels. YouTube and Google Business disconnected. Pinterest skipped.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2148,32 +1710,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>perfect-meeting-danger, perfect-meeting-fix</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>8, 8</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Pain point topic. YouTube/Google Business disconnected. TikTok scheduled May 25-26.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2190,32 +1727,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>learning-leader-rec, learning-leader-lessons</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>8, 8</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Podcast rec for Ryan Hawk. YouTube/Google Business disconnected. TikTok scheduled May 27-28.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2232,30 +1744,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="n">
-        <v>46108</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>offsite-insights-edward-amey, leadership-disability-edward-amey</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>8, 7</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>No specific testimonial quote found. Built carousels from verified podcast content (EP225) and public bio.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2272,30 +1761,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="n">
-        <v>46108</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>why-leaders-need-a-coach, what-coaching-looks-like, cost-of-no-coach</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>8, 8, 8</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>Service promo carousel. No people tagged.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2312,32 +1778,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>wg-6-types, wg-genius-or-frustration, wg-transforms-teams</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>8, 8, 8</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>All 9 platforms scheduled. YouTube on Apr 15-17 due to daily limits.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2354,32 +1795,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>5d-overview, 5d-overcome, 5d-warning-signs</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>8, 8, 8</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>All 9 platforms scheduled. YouTube on Apr 18-20.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2396,32 +1812,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>crucial-conversations-why-read, crucial-conversations-7-skills, crucial-conversations-apply</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>8, 9, 8</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>Book rec. 3 carousels. All 9 platforms. YouTube Apr 28-30. TikTok Jun 9-11. Pinterest skipped (no boards).</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2438,32 +1829,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>teacher-resigned-what-happened, teacher-resigned-warning-signs, teacher-resigned-how-to-keep</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>8, 8, 8</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Pain point. 3 carousels. All 9 platforms. YouTube May 1-3. TikTok Jun 12-14. Pinterest skipped.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2480,32 +1846,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>dare-to-lead-why-listen, dare-to-lead-key-themes</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>8, 7</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>Podcast rec. 2 carousels. All 9 platforms. YouTube May 4-5. TikTok Jun 15-16. Pinterest skipped.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2522,12 +1863,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Skipped</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>No testimonial content found online. Needs manual input of testimonial text.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2544,32 +1880,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>board-offsite-why, board-offsite-5-signs</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>8, 7</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Service topic. No blog URL. 2 carousels. Tim Chalmers row skipped (no content found).</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2586,32 +1897,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>pre-brief-call, 5-questions-before-offsite</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>8, 8</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>Behind the scenes content. No people to tag.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2621,11 +1907,6 @@
           <t>Vulnerability-Based Trust</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
-        </is>
-      </c>
       <c r="D54" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2633,32 +1914,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>what-is-vulnerability-based-trust, 7-ways-vulnerability-trust, leader-must-go-first</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>8, 9, 8</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>Blog post carousel. 3 carousels from Lencioni VBT concept.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2675,32 +1931,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>atomic-habits-book-rec, 4-laws-behaviour-change</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>8, 8</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>Book rec. James Clear tagged. Footer: Author | Keynote Speaker</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2717,27 +1948,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>offsite-nothing-changed, 3-signs-offsite-fail</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>8, 7</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2118,32 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>school-pd-book-jonno, school-pd-great-day, school-pd-reasons</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>7, 8, 7</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Education footer. 3 carousels. ASBA 2025 stats referenced.</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2160,32 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>step-up-framework, step-up-expectations</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>2 carousels. 10,000+ copies referenced. No fabricated testimonials.</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2202,32 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>personal-histories-exercise, personal-histories-why</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>2 carousels. Patrick Lencioni tagged. Five Dysfunctions referenced.</t>
         </is>
       </c>
     </row>
@@ -2958,7 +2244,32 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>ideal-team-player-why, ideal-team-player-missing</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>2 carousels. Humble/Hungry/Smart framework. Lencioni tagged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - 2026-03-27 run
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -59,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1370,7 +1373,32 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Why Listen to Craig Groeschel, 5 Key Themes, 3 Reasons to Subscribe</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>8, 7, 6</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Pinterest skipped (no boards)</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1415,32 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>asba-working-genius-in-action, asba-93-percent-rated-excellent, asba-what-school-leaders-took-away</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>7, 7, 7</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>3 carousels from ASBA testimonial. TikTok/YouTube hit daily Buffer limits. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1457,32 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>offsite-why-your-team-needs-one, offsite-what-to-expect, offsite-common-mistakes, offsite-book-your-offsite</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>8, 8, 8, 7</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>4 carousels from service page. Pinterest skipped (no boards). YouTube Apr 11-14. TikTok May 8-11.</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1499,32 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>5-dysfunctions-overview, 5-dysfunctions-trust-conflict, 5-dysfunctions-commitment-results, 5-dysfunctions-action-plan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>9, 8, 9, 8</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>4 carousels from framework topic. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1541,32 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>imposter-syndrome-signs, imposter-syndrome-cost, imposter-syndrome-overcome</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>3 carousels from blog topic. Pinterest skipped.</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1583,32 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>unreasonable-hospitality-why-read, unreasonable-hospitality-lessons, unreasonable-hospitality-apply</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>7, 7, 7</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>3 carousels from book rec. Pinterest skipped.</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1625,32 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>losing-teachers-warning-signs, losing-teachers-real-reasons, losing-teachers-what-to-do</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>8, 8, 7</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>3 carousels from pain point topic. Pinterest skipped.</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1667,32 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>hbr-ideacast-why-listen, hbr-ideacast-key-themes, hbr-ideacast-reasons-subscribe</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>8, 7, 6</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>3 carousels from podcast rec. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1709,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>redlands-wg-overview, redlands-wg-discoveries, redlands-wg-book-session</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1736,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>schools-wg-why, schools-wg-how, schools-wg-transform</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1763,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>wg-session-inside, wg-session-moments, wg-session-book</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1790,32 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>understanding-uncertainty, decision-making-uncertainty, communication-trust-uncertainty, resilience-adaptive-strategy</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>8, 8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>4 carousels from blog post. All 9 platforms scheduled. YouTube Apr 15-18. TikTok Mar 30-31.</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1832,32 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>radical-candor-why-read, radical-candor-four-quadrants, radical-candor-in-practice</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>3 carousels from book rec. All 9 platforms. YouTube Apr 19-21. TikTok Apr 1-2.</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1874,32 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>why-priorities-fail, signs-plan-will-fail, break-the-cycle</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>8, 7, 8</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky (carousel 3: 5 platforms failed duplicate detection)</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Pain point topic. 3 carousels. Carousel 3 blocked by Buffer duplicate detection on LI/FB/Threads/X/Bluesky.</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1916,32 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>worklife-podcast-rec, worklife-why-listen</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2 carousels. All 9 platforms scheduled successfully.</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1958,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>No testimonial content found online. Needs manual input of testimonial text.</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1980,32 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>keynote-speaking-service, why-book-jonno</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2 carousels. All 9 platforms scheduled successfully.</t>
         </is>
       </c>
     </row>
@@ -1659,7 +2022,32 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>asba-93-percent-proof, asba-what-makes-pd-great</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2 carousels. YouTube and Google Business disconnected. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>
@@ -1676,7 +2064,32 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>exec-team-dysfunction, fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>9, 7</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2 carousels. All 9 platforms scheduled successfully. Based on Lencioni's Five Dysfunctions.</t>
         </is>
       </c>
     </row>
@@ -1693,7 +2106,32 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>extreme-ownership-why-read, extreme-ownership-principles, extreme-ownership-apply</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>8, 8, 7</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>3 carousels. YouTube and Google Business disconnected. Pinterest skipped.</t>
         </is>
       </c>
     </row>
@@ -1710,7 +2148,32 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>perfect-meeting-danger, perfect-meeting-fix</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Pain point topic. YouTube/Google Business disconnected. TikTok scheduled May 25-26.</t>
         </is>
       </c>
     </row>
@@ -1727,7 +2190,32 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>learning-leader-rec, learning-leader-lessons</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Podcast rec for Ryan Hawk. YouTube/Google Business disconnected. TikTok scheduled May 27-28.</t>
         </is>
       </c>
     </row>
@@ -1744,7 +2232,30 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>offsite-insights-edward-amey, leadership-disability-edward-amey</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>No specific testimonial quote found. Built carousels from verified podcast content (EP225) and public bio.</t>
         </is>
       </c>
     </row>
@@ -1761,7 +2272,30 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>why-leaders-need-a-coach, what-coaching-looks-like, cost-of-no-coach</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Service promo carousel. No people tagged.</t>
         </is>
       </c>
     </row>
@@ -1778,7 +2312,32 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>wg-6-types, wg-genius-or-frustration, wg-transforms-teams</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>All 9 platforms scheduled. YouTube on Apr 15-17 due to daily limits.</t>
         </is>
       </c>
     </row>
@@ -1795,7 +2354,32 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>5d-overview, 5d-overcome, 5d-warning-signs</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>All 9 platforms scheduled. YouTube on Apr 18-20.</t>
         </is>
       </c>
     </row>
@@ -1812,7 +2396,32 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>crucial-conversations-why-read, crucial-conversations-7-skills, crucial-conversations-apply</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>8, 9, 8</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Book rec. 3 carousels. All 9 platforms. YouTube Apr 28-30. TikTok Jun 9-11. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>
@@ -1829,7 +2438,32 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>teacher-resigned-what-happened, teacher-resigned-warning-signs, teacher-resigned-how-to-keep</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Pain point. 3 carousels. All 9 platforms. YouTube May 1-3. TikTok Jun 12-14. Pinterest skipped.</t>
         </is>
       </c>
     </row>
@@ -1846,7 +2480,32 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>dare-to-lead-why-listen, dare-to-lead-key-themes</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Podcast rec. 2 carousels. All 9 platforms. YouTube May 4-5. TikTok Jun 15-16. Pinterest skipped.</t>
         </is>
       </c>
     </row>
@@ -1863,7 +2522,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>No testimonial content found online. Needs manual input of testimonial text.</t>
         </is>
       </c>
     </row>
@@ -1880,7 +2544,32 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>board-offsite-why, board-offsite-5-signs</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Service topic. No blog URL. 2 carousels. Tim Chalmers row skipped (no content found).</t>
         </is>
       </c>
     </row>
@@ -1897,7 +2586,32 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>pre-brief-call, 5-questions-before-offsite</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Behind the scenes content. No people to tag.</t>
         </is>
       </c>
     </row>
@@ -1907,6 +2621,11 @@
           <t>Vulnerability-Based Trust</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1914,7 +2633,32 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>what-is-vulnerability-based-trust, 7-ways-vulnerability-trust, leader-must-go-first</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>8, 9, 8</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Blog post carousel. 3 carousels from Lencioni VBT concept.</t>
         </is>
       </c>
     </row>
@@ -1931,7 +2675,32 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>atomic-habits-book-rec, 4-laws-behaviour-change</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Book rec. James Clear tagged. Footer: Author | Keynote Speaker</t>
         </is>
       </c>
     </row>
@@ -1948,7 +2717,32 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>offsite-why-nothing-changed, offsite-how-to-stick</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Pain point topic. No blog URL. Content researched via web search.</t>
         </is>
       </c>
     </row>
@@ -1965,7 +2759,32 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>maxwell-podcast-why-listen, maxwell-podcast-key-themes</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Podcast rec. TikTok Jun 21, YouTube Jun 12.</t>
         </is>
       </c>
     </row>
@@ -1982,7 +2801,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>No testimonial quote found via web search. Cannot fabricate quotes per workflow rules.</t>
         </is>
       </c>
     </row>
@@ -1999,7 +2823,32 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>strategic-plan-why-facilitator, strategic-plan-5-signs-dust</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Service topic. TikTok Jun 22-23, YouTube Jun 13-14.</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2865,32 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>step-up-10k-milestone, step-up-3-stages</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Book milestone. TikTok Jun 24-25, YouTube Jun 15-16.</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2907,32 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>build-relationships-first, avoid-common-mistakes, lead-instruction-with-confidence</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>No blog URL. Content researched from web. School topic, used WG Facilitator footer.</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2949,32 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>why-read-hidden-potential, key-ideas-hidden-potential, apply-hidden-potential</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>8, 7, 7</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Book Rec. Adam Grant tagged on IG (@adamgrant) and X (@AdamMGrant).</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2991,32 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>signs-of-team-dysfunction, root-causes-team-dysfunction, fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>9, 7, 8</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Pain Point topic. No people featured (advice content). TikTok on Apr 2-3, YouTube on May 2-4.</t>
         </is>
       </c>
     </row>
@@ -2084,7 +3033,32 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>why-listen-coaching-for-leaders, best-episodes-coaching-for-leaders, lessons-from-coaching-for-leaders</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>7, 8, 7</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Podcast Rec. Dave Stachowiak tagged on X (@davestachowiak). TikTok on Apr 3-4, YouTube on May 5-7.</t>
         </is>
       </c>
     </row>
@@ -2101,7 +3075,12 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Testimonial text not found on website. Needs manual input.</t>
         </is>
       </c>
     </row>
@@ -2128,22 +3107,22 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>school-pd-book-jonno, school-pd-great-day, school-pd-reasons</t>
+          <t>school-pd-day-what-2026-03-27, school-pd-day-why-2026-03-27</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>7, 8, 7</t>
+          <t>8, 8</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube*, Bluesky</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Education footer. 3 carousels. ASBA 2025 stats referenced.</t>
+          <t>YouTube logged for manual upload (queue full)</t>
         </is>
       </c>
     </row>
@@ -2170,7 +3149,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>step-up-framework, step-up-expectations</t>
+          <t>step-up-framework-2026-03-27, step-up-signs-2026-03-27</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -2180,12 +3159,12 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+          <t>LinkedIn*, Facebook*, Instagram, Threads*, X/Twitter*, Google Business, TikTok, YouTube*, Bluesky</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2 carousels. 10,000+ copies referenced. No fabricated testimonials.</t>
+          <t>Some platforms rejected carousel 2A as duplicate. YouTube queue full. *=partial</t>
         </is>
       </c>
     </row>
@@ -2212,22 +3191,22 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>personal-histories-exercise, personal-histories-why</t>
+          <t>personal-histories-2026-03-27, personal-histories-how-2026-03-27</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>8, 7</t>
+          <t>8, 8</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube*, Bluesky</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2 carousels. Patrick Lencioni tagged. Five Dysfunctions referenced.</t>
+          <t>YouTube logged for manual upload (queue full)</t>
         </is>
       </c>
     </row>
@@ -2254,22 +3233,22 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>ideal-team-player-why, ideal-team-player-missing</t>
+          <t>ideal-team-player-2026-03-27</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>8, 8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube*, Bluesky</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>2 carousels. Humble/Hungry/Smart framework. Lencioni tagged.</t>
+          <t>YouTube logged for manual upload (queue full)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar — 4 topics scheduled 2026-03-27
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -3080,7 +3080,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Testimonial text not found on website. Needs manual input.</t>
+          <t>Testimonial text not found online. Cannot fabricate.</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3107,22 +3107,22 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>school-pd-day-what-2026-03-27, school-pd-day-why-2026-03-27</t>
+          <t>school-pd-day-reasons, school-pd-day-agenda</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>8, 8</t>
+          <t>7, 8</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube*, Bluesky</t>
+          <t>LI, FB, IG, Threads, X, GBP, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>YouTube logged for manual upload (queue full)</t>
+          <t>Service carousel. 9 platforms each.</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>step-up-framework-2026-03-27, step-up-signs-2026-03-27</t>
+          <t>step-up-framework, step-up-signs</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3159,12 +3159,12 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>LinkedIn*, Facebook*, Instagram, Threads*, X/Twitter*, Google Business, TikTok, YouTube*, Bluesky</t>
+          <t>LI, FB, IG, Threads, X, GBP, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Some platforms rejected carousel 2A as duplicate. YouTube queue full. *=partial</t>
+          <t>Framework carousel. 9 platforms each.</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3191,22 +3191,22 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>personal-histories-2026-03-27, personal-histories-how-2026-03-27</t>
+          <t>personal-histories-what, personal-histories-why</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>8, 8</t>
+          <t>8, 7</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube*, Bluesky</t>
+          <t>LI, FB, IG, Threads, X, GBP, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>YouTube logged for manual upload (queue full)</t>
+          <t>Blog carousel. 9 platforms each.</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3233,22 +3233,22 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>ideal-team-player-2026-03-27</t>
+          <t>ideal-team-player-book, ideal-team-player-missing</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8, 8</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube*, Bluesky</t>
+          <t>LI, FB, IG, Threads, X, GBP, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>YouTube logged for manual upload (queue full)</t>
+          <t>Book rec carousel. 9 platforms each.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - rows 65-69 processed (2026-03-27 session 2)
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -3080,7 +3080,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Testimonial text not found online. Cannot fabricate.</t>
+          <t>No verifiable testimonial found online. Skipped per rule: never fabricate quotes.</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Carousel Created</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3107,22 +3107,22 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>school-pd-day-reasons, school-pd-day-agenda</t>
+          <t>what-a-pd-day-looks-like, why-book-jonno-pd-day</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>7, 8</t>
+          <t>8, 7</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>LI, FB, IG, Threads, X, GBP, Bluesky, TikTok, YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Service carousel. 9 platforms each.</t>
+          <t>School topic. Role: Certified Working Genius Facilitator | Author</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Carousel Created</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>step-up-framework, step-up-signs</t>
+          <t>step-up-step-out-framework, 5-signs-have-conversation</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3159,12 +3159,12 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>LI, FB, IG, Threads, X, GBP, Bluesky, TikTok, YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Framework carousel. 9 platforms each.</t>
+          <t>Framework topic.</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Carousel Created</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>personal-histories-what, personal-histories-why</t>
+          <t>build-trust-30-minutes, how-to-run-personal-histories</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3201,12 +3201,12 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>LI, FB, IG, Threads, X, GBP, Bluesky, TikTok, YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Blog carousel. 9 platforms each.</t>
+          <t>Trust-building exercise topic.</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Carousel Created</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3233,22 +3233,22 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>ideal-team-player-book, ideal-team-player-missing</t>
+          <t>ideal-team-player-book, are-you-ideal-team-player</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>8, 8</t>
+          <t>8, 7</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>LI, FB, IG, Threads, X, GBP, Bluesky, TikTok, YouTube</t>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Book rec carousel. 9 platforms each.</t>
+          <t>Book Rec. Patrick Lencioni.</t>
         </is>
       </c>
     </row>

</xml_diff>